<commit_message>
feat: Sample data for olivine
</commit_message>
<xml_diff>
--- a/demo-data/olivine_demo_3rd_party.xlsx
+++ b/demo-data/olivine_demo_3rd_party.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -488,7 +488,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>08.10.26</t>
+          <t>27.09.26</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>6681</v>
+        <v>4407</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -525,13 +525,13 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>585.11</v>
+        <v>465.09</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>11.10.26</t>
+          <t>05.09.26</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -555,7 +555,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>7561</v>
+        <v>9632</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -568,13 +568,13 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>308.81</v>
+        <v>412.59</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>12.10.26</t>
+          <t>24.09.26</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>16773</v>
+        <v>15227</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -611,13 +611,13 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>203.79</v>
+        <v>552.2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>17.10.26</t>
+          <t>14.09.26</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>4361</v>
+        <v>16956</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -654,13 +654,13 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>219.36</v>
+        <v>122.33</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>19.10.26</t>
+          <t>28.09.26</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -684,7 +684,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>11690</v>
+        <v>6636</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -697,13 +697,13 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>509.14</v>
+        <v>241.4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>23.10.26</t>
+          <t>18.09.26</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>10718</v>
+        <v>4350</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -740,13 +740,13 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>193.66</v>
+        <v>359.36</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>21.10.26</t>
+          <t>28.09.26</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>9435</v>
+        <v>12235</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -783,13 +783,13 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>479.54</v>
+        <v>251.49</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>13.10.26</t>
+          <t>03.08.26</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -813,7 +813,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>14217</v>
+        <v>8699</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -826,13 +826,13 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>341.74</v>
+        <v>439.17</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04.10.26</t>
+          <t>23.09.26</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -856,7 +856,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>12285</v>
+        <v>15985</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -869,13 +869,13 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>363.14</v>
+        <v>612.62</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>20.10.26</t>
+          <t>07.08.26</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -899,7 +899,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>5508</v>
+        <v>7078</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -912,13 +912,13 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>469.11</v>
+        <v>545.8099999999999</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>05.10.26</t>
+          <t>28.09.26</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -942,7 +942,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>10915</v>
+        <v>7373</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -955,13 +955,13 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>649.52</v>
+        <v>527.5599999999999</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>07.10.26</t>
+          <t>29.08.26</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>9927</v>
+        <v>8980</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -998,13 +998,13 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>189.43</v>
+        <v>328.15</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>24.10.26</t>
+          <t>24.09.26</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1028,7 +1028,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>14205</v>
+        <v>14841</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1041,13 +1041,13 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>249.53</v>
+        <v>95.42</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>03.10.26</t>
+          <t>28.09.26</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1071,7 +1071,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>10795</v>
+        <v>15005</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1084,13 +1084,13 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>99.11</v>
+        <v>551.45</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>22.10.26</t>
+          <t>26.09.26</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1114,7 +1114,7 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>16542</v>
+        <v>13351</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1127,13 +1127,13 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>406.44</v>
+        <v>284.94</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>05.10.26</t>
+          <t>13.08.26</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>10136</v>
+        <v>11096</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1170,13 +1170,13 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>465.72</v>
+        <v>468.29</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>02.10.26</t>
+          <t>27.09.26</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1200,7 +1200,7 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>16200</v>
+        <v>14925</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1213,13 +1213,13 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>343.05</v>
+        <v>220.63</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>06.10.26</t>
+          <t>22.08.26</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1243,7 +1243,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>10634</v>
+        <v>14976</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1256,13 +1256,13 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>638.95</v>
+        <v>226.11</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>15.10.26</t>
+          <t>26.09.26</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1286,7 +1286,7 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>12148</v>
+        <v>4009</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1299,13 +1299,13 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>228.44</v>
+        <v>357.59</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>13.10.26</t>
+          <t>22.09.26</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1329,7 +1329,7 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>6680</v>
+        <v>14179</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1342,13 +1342,13 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>207.17</v>
+        <v>496.86</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>07.10.26</t>
+          <t>22.09.26</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1372,7 +1372,7 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>11966</v>
+        <v>9909</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1385,13 +1385,13 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>515.1</v>
+        <v>99.15000000000001</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>11.10.26</t>
+          <t>30.08.26</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1415,7 +1415,7 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>10133</v>
+        <v>14124</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1428,13 +1428,13 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>154.32</v>
+        <v>140.63</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>06.10.26</t>
+          <t>26.09.26</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1477,7 +1477,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>06.10.26</t>
+          <t>26.09.26</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1520,7 +1520,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12.10.26</t>
+          <t>25.09.26</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1555,6 +1555,135 @@
         <is>
           <t>Bulawayo</t>
         </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>28.09.26</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Hypery</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Bakers Inn Bakeries</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>ZEE TRUCKING</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>INV-9100</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>9200</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>ABC7788</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Harare</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>28.09.26</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Olivine</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Brainscope</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>SIGHTSCORE</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>INV-9101</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>5400</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>AGL8230</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Gweru</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>265.5</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>27.09.26</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Surface</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Kingy Wholesalers</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>NORTHLAND</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>INV-9102</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>7100</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>AGJ7091</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Masvingo</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>410.75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>